<commit_message>
Working on including inverters
</commit_message>
<xml_diff>
--- a/microgridspy/results/Costs Breakdown.xlsx
+++ b/microgridspy/results/Costs Breakdown.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Cost Item</t>
   </si>
@@ -40,46 +40,22 @@
     <t>Total Salvage Value (Actualized)</t>
   </si>
   <si>
-    <t>Grid Investment Cost (Actualized)</t>
-  </si>
-  <si>
-    <t>Grid Fixed O&amp;M Cost (Actualized)</t>
-  </si>
-  <si>
-    <t>Total Electricity Purchased Cost (Actualized)</t>
-  </si>
-  <si>
-    <t>Total Electricity Sold Revenue (Actualized)</t>
-  </si>
-  <si>
-    <t>8921.75</t>
-  </si>
-  <si>
-    <t>7007.08</t>
-  </si>
-  <si>
-    <t>2609.30</t>
-  </si>
-  <si>
-    <t>729.18</t>
-  </si>
-  <si>
-    <t>3502.68</t>
-  </si>
-  <si>
-    <t>20.81</t>
-  </si>
-  <si>
-    <t>140.00</t>
-  </si>
-  <si>
-    <t>3.50</t>
-  </si>
-  <si>
-    <t>266.02</t>
-  </si>
-  <si>
-    <t>100.09</t>
+    <t>72.73</t>
+  </si>
+  <si>
+    <t>9.60</t>
+  </si>
+  <si>
+    <t>4.25</t>
+  </si>
+  <si>
+    <t>1.51</t>
+  </si>
+  <si>
+    <t>3.83</t>
+  </si>
+  <si>
+    <t>53.58</t>
   </si>
 </sst>
 </file>
@@ -437,7 +413,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -453,7 +429,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -461,7 +437,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -469,7 +445,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -477,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -485,7 +461,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -493,39 +469,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved plots dashboard and grid page
</commit_message>
<xml_diff>
--- a/microgridspy/results/Costs Breakdown.xlsx
+++ b/microgridspy/results/Costs Breakdown.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Cost Item</t>
   </si>
@@ -31,25 +31,49 @@
     <t xml:space="preserve"> - Total Fixed O&amp;M Cost (Actualized)</t>
   </si>
   <si>
+    <t xml:space="preserve"> - Total Battery Replacement Cost (Actualized)</t>
+  </si>
+  <si>
     <t xml:space="preserve"> - Total Fuel Cost (Actualized)</t>
   </si>
   <si>
     <t>Total Salvage Value (Actualized)</t>
   </si>
   <si>
-    <t>43.10</t>
-  </si>
-  <si>
-    <t>295.66</t>
-  </si>
-  <si>
-    <t>7.62</t>
-  </si>
-  <si>
-    <t>288.05</t>
-  </si>
-  <si>
-    <t>8.31</t>
+    <t>Grid Investment Cost (Actualized)</t>
+  </si>
+  <si>
+    <t>Grid Fixed O&amp;M Cost (Actualized)</t>
+  </si>
+  <si>
+    <t>Total Electricity Purchased Cost (Actualized)</t>
+  </si>
+  <si>
+    <t>1822.90</t>
+  </si>
+  <si>
+    <t>4203.31</t>
+  </si>
+  <si>
+    <t>516.82</t>
+  </si>
+  <si>
+    <t>117.08</t>
+  </si>
+  <si>
+    <t>2976.94</t>
+  </si>
+  <si>
+    <t>8.33</t>
+  </si>
+  <si>
+    <t>96.00</t>
+  </si>
+  <si>
+    <t>2.40</t>
+  </si>
+  <si>
+    <t>592.47</t>
   </si>
 </sst>
 </file>
@@ -407,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -423,7 +447,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -431,7 +455,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -439,7 +463,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -447,7 +471,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -455,7 +479,39 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>